<commit_message>
Update product import file with correct quantities
Correctly includes actual product quantities in the generated XLSX file, overwriting the previously applied default of zero.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: d8b59655-72ed-42b1-b048-a1920ad7692a
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: e8b24b01-f83b-4358-9543-162d6bc283bd
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/attached_assets/products_handwritten_import_ready.xlsx
+++ b/attached_assets/products_handwritten_import_ready.xlsx
@@ -469,7 +469,7 @@
         <v/>
       </c>
       <c r="H2">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="I2" t="str">
         <v/>
@@ -516,7 +516,7 @@
         <v/>
       </c>
       <c r="H3">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="I3" t="str">
         <v/>
@@ -563,7 +563,7 @@
         <v/>
       </c>
       <c r="H4">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="I4" t="str">
         <v/>
@@ -610,7 +610,7 @@
         <v/>
       </c>
       <c r="H5">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="I5" t="str">
         <v/>
@@ -657,7 +657,7 @@
         <v/>
       </c>
       <c r="H6">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="I6" t="str">
         <v/>
@@ -704,7 +704,7 @@
         <v/>
       </c>
       <c r="H7">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="I7" t="str">
         <v/>
@@ -751,7 +751,7 @@
         <v/>
       </c>
       <c r="H8">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="I8" t="str">
         <v/>
@@ -798,7 +798,7 @@
         <v/>
       </c>
       <c r="H9">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="I9" t="str">
         <v/>
@@ -845,7 +845,7 @@
         <v/>
       </c>
       <c r="H10">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I10" t="str">
         <v/>
@@ -892,7 +892,7 @@
         <v/>
       </c>
       <c r="H11">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I11" t="str">
         <v/>
@@ -939,7 +939,7 @@
         <v/>
       </c>
       <c r="H12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I12" t="str">
         <v/>
@@ -986,7 +986,7 @@
         <v/>
       </c>
       <c r="H13">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I13" t="str">
         <v/>
@@ -1033,7 +1033,7 @@
         <v/>
       </c>
       <c r="H14">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I14" t="str">
         <v/>
@@ -1080,7 +1080,7 @@
         <v/>
       </c>
       <c r="H15">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I15" t="str">
         <v/>
@@ -1127,7 +1127,7 @@
         <v/>
       </c>
       <c r="H16">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I16" t="str">
         <v/>
@@ -1174,7 +1174,7 @@
         <v/>
       </c>
       <c r="H17">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I17" t="str">
         <v/>
@@ -1221,7 +1221,7 @@
         <v/>
       </c>
       <c r="H18">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I18" t="str">
         <v/>
@@ -1268,7 +1268,7 @@
         <v/>
       </c>
       <c r="H19">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I19" t="str">
         <v/>
@@ -1315,7 +1315,7 @@
         <v/>
       </c>
       <c r="H20">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="I20" t="str">
         <v/>
@@ -1362,7 +1362,7 @@
         <v/>
       </c>
       <c r="H21">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="I21" t="str">
         <v/>
@@ -1409,7 +1409,7 @@
         <v/>
       </c>
       <c r="H22">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="I22" t="str">
         <v/>
@@ -1456,7 +1456,7 @@
         <v/>
       </c>
       <c r="H23">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I23" t="str">
         <v/>
@@ -1503,7 +1503,7 @@
         <v/>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="I24" t="str">
         <v/>
@@ -1550,7 +1550,7 @@
         <v/>
       </c>
       <c r="H25">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="I25" t="str">
         <v/>
@@ -1597,7 +1597,7 @@
         <v/>
       </c>
       <c r="H26">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I26" t="str">
         <v/>
@@ -1644,7 +1644,7 @@
         <v/>
       </c>
       <c r="H27">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I27" t="str">
         <v/>
@@ -1691,7 +1691,7 @@
         <v/>
       </c>
       <c r="H28">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="I28" t="str">
         <v/>
@@ -1738,7 +1738,7 @@
         <v/>
       </c>
       <c r="H29">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="I29" t="str">
         <v/>
@@ -1785,7 +1785,7 @@
         <v/>
       </c>
       <c r="H30">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="I30" t="str">
         <v/>
@@ -1832,7 +1832,7 @@
         <v/>
       </c>
       <c r="H31">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="I31" t="str">
         <v/>
@@ -1879,7 +1879,7 @@
         <v/>
       </c>
       <c r="H32">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="I32" t="str">
         <v/>
@@ -1926,7 +1926,7 @@
         <v/>
       </c>
       <c r="H33">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I33" t="str">
         <v/>
@@ -1973,7 +1973,7 @@
         <v/>
       </c>
       <c r="H34">
-        <v>0</v>
+        <v>92</v>
       </c>
       <c r="I34" t="str">
         <v/>
@@ -2020,7 +2020,7 @@
         <v/>
       </c>
       <c r="H35">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="I35" t="str">
         <v/>
@@ -2067,7 +2067,7 @@
         <v/>
       </c>
       <c r="H36">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I36" t="str">
         <v/>
@@ -2114,7 +2114,7 @@
         <v/>
       </c>
       <c r="H37">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I37" t="str">
         <v/>
@@ -2161,7 +2161,7 @@
         <v/>
       </c>
       <c r="H38">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="I38" t="str">
         <v/>
@@ -2208,7 +2208,7 @@
         <v/>
       </c>
       <c r="H39">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I39" t="str">
         <v/>
@@ -2255,7 +2255,7 @@
         <v/>
       </c>
       <c r="H40">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="I40" t="str">
         <v/>
@@ -2302,7 +2302,7 @@
         <v/>
       </c>
       <c r="H41">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I41" t="str">
         <v/>
@@ -2349,7 +2349,7 @@
         <v/>
       </c>
       <c r="H42">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I42" t="str">
         <v/>
@@ -2396,7 +2396,7 @@
         <v/>
       </c>
       <c r="H43">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="I43" t="str">
         <v/>
@@ -2443,7 +2443,7 @@
         <v/>
       </c>
       <c r="H44">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I44" t="str">
         <v/>
@@ -2490,7 +2490,7 @@
         <v/>
       </c>
       <c r="H45">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I45" t="str">
         <v/>
@@ -2537,7 +2537,7 @@
         <v/>
       </c>
       <c r="H46">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I46" t="str">
         <v/>
@@ -2584,7 +2584,7 @@
         <v/>
       </c>
       <c r="H47">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I47" t="str">
         <v/>
@@ -2631,7 +2631,7 @@
         <v/>
       </c>
       <c r="H48">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I48" t="str">
         <v/>
@@ -2678,7 +2678,7 @@
         <v/>
       </c>
       <c r="H49">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="I49" t="str">
         <v/>
@@ -2725,7 +2725,7 @@
         <v/>
       </c>
       <c r="H50">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I50" t="str">
         <v/>
@@ -2772,7 +2772,7 @@
         <v/>
       </c>
       <c r="H51">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I51" t="str">
         <v/>
@@ -2819,7 +2819,7 @@
         <v/>
       </c>
       <c r="H52">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I52" t="str">
         <v/>
@@ -2866,7 +2866,7 @@
         <v/>
       </c>
       <c r="H53">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I53" t="str">
         <v/>
@@ -2913,7 +2913,7 @@
         <v/>
       </c>
       <c r="H54">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I54" t="str">
         <v/>
@@ -2960,7 +2960,7 @@
         <v/>
       </c>
       <c r="H55">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="I55" t="str">
         <v/>
@@ -3007,7 +3007,7 @@
         <v/>
       </c>
       <c r="H56">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="I56" t="str">
         <v/>
@@ -3054,7 +3054,7 @@
         <v/>
       </c>
       <c r="H57">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="I57" t="str">
         <v/>
@@ -3101,7 +3101,7 @@
         <v/>
       </c>
       <c r="H58">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I58" t="str">
         <v/>
@@ -3148,7 +3148,7 @@
         <v/>
       </c>
       <c r="H59">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="I59" t="str">
         <v/>
@@ -3195,7 +3195,7 @@
         <v/>
       </c>
       <c r="H60">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I60" t="str">
         <v/>
@@ -3242,7 +3242,7 @@
         <v/>
       </c>
       <c r="H61">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I61" t="str">
         <v/>
@@ -3289,7 +3289,7 @@
         <v/>
       </c>
       <c r="H62">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I62" t="str">
         <v/>
@@ -3336,7 +3336,7 @@
         <v/>
       </c>
       <c r="H63">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="I63" t="str">
         <v/>
@@ -3383,7 +3383,7 @@
         <v/>
       </c>
       <c r="H64">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I64" t="str">
         <v/>
@@ -3430,7 +3430,7 @@
         <v/>
       </c>
       <c r="H65">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="I65" t="str">
         <v/>
@@ -3477,7 +3477,7 @@
         <v/>
       </c>
       <c r="H66">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I66" t="str">
         <v/>
@@ -3524,7 +3524,7 @@
         <v/>
       </c>
       <c r="H67">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I67" t="str">
         <v/>
@@ -3571,7 +3571,7 @@
         <v/>
       </c>
       <c r="H68">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I68" t="str">
         <v/>
@@ -3618,7 +3618,7 @@
         <v/>
       </c>
       <c r="H69">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I69" t="str">
         <v/>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="H70">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I70" t="str">
         <v/>
@@ -3712,7 +3712,7 @@
         <v/>
       </c>
       <c r="H71">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="I71" t="str">
         <v/>
@@ -3759,7 +3759,7 @@
         <v/>
       </c>
       <c r="H72">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I72" t="str">
         <v/>
@@ -3806,7 +3806,7 @@
         <v/>
       </c>
       <c r="H73">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I73" t="str">
         <v/>
@@ -3853,7 +3853,7 @@
         <v/>
       </c>
       <c r="H74">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I74" t="str">
         <v/>
@@ -3900,7 +3900,7 @@
         <v/>
       </c>
       <c r="H75">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I75" t="str">
         <v/>
@@ -3947,7 +3947,7 @@
         <v/>
       </c>
       <c r="H76">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="I76" t="str">
         <v/>
@@ -3994,7 +3994,7 @@
         <v/>
       </c>
       <c r="H77">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I77" t="str">
         <v/>
@@ -4041,7 +4041,7 @@
         <v/>
       </c>
       <c r="H78">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I78" t="str">
         <v/>
@@ -4088,7 +4088,7 @@
         <v/>
       </c>
       <c r="H79">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I79" t="str">
         <v/>
@@ -4135,7 +4135,7 @@
         <v/>
       </c>
       <c r="H80">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I80" t="str">
         <v/>
@@ -4182,7 +4182,7 @@
         <v/>
       </c>
       <c r="H81">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I81" t="str">
         <v/>
@@ -4229,7 +4229,7 @@
         <v/>
       </c>
       <c r="H82">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I82" t="str">
         <v/>
@@ -4276,7 +4276,7 @@
         <v/>
       </c>
       <c r="H83">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="I83" t="str">
         <v/>
@@ -4323,7 +4323,7 @@
         <v/>
       </c>
       <c r="H84">
-        <v>0</v>
+        <v>79</v>
       </c>
       <c r="I84" t="str">
         <v/>
@@ -4370,7 +4370,7 @@
         <v/>
       </c>
       <c r="H85">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="I85" t="str">
         <v/>
@@ -4417,7 +4417,7 @@
         <v/>
       </c>
       <c r="H86">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I86" t="str">
         <v/>
@@ -4464,7 +4464,7 @@
         <v/>
       </c>
       <c r="H87">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I87" t="str">
         <v/>
@@ -4511,7 +4511,7 @@
         <v/>
       </c>
       <c r="H88">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="I88" t="str">
         <v/>
@@ -4558,7 +4558,7 @@
         <v/>
       </c>
       <c r="H89">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="I89" t="str">
         <v/>
@@ -4605,7 +4605,7 @@
         <v/>
       </c>
       <c r="H90">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="I90" t="str">
         <v/>
@@ -4652,7 +4652,7 @@
         <v/>
       </c>
       <c r="H91">
-        <v>0</v>
+        <v>44</v>
       </c>
       <c r="I91" t="str">
         <v/>
@@ -4699,7 +4699,7 @@
         <v/>
       </c>
       <c r="H92">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I92" t="str">
         <v/>
@@ -4746,7 +4746,7 @@
         <v/>
       </c>
       <c r="H93">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I93" t="str">
         <v/>
@@ -4793,7 +4793,7 @@
         <v/>
       </c>
       <c r="H94">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I94" t="str">
         <v/>
@@ -4840,7 +4840,7 @@
         <v/>
       </c>
       <c r="H95">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I95" t="str">
         <v/>
@@ -4887,7 +4887,7 @@
         <v/>
       </c>
       <c r="H96">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I96" t="str">
         <v/>
@@ -4934,7 +4934,7 @@
         <v/>
       </c>
       <c r="H97">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I97" t="str">
         <v/>
@@ -4981,7 +4981,7 @@
         <v/>
       </c>
       <c r="H98">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="I98" t="str">
         <v/>
@@ -5028,7 +5028,7 @@
         <v/>
       </c>
       <c r="H99">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="I99" t="str">
         <v/>
@@ -5075,7 +5075,7 @@
         <v/>
       </c>
       <c r="H100">
-        <v>0</v>
+        <v>66</v>
       </c>
       <c r="I100" t="str">
         <v/>
@@ -5122,7 +5122,7 @@
         <v/>
       </c>
       <c r="H101">
-        <v>0</v>
+        <v>77</v>
       </c>
       <c r="I101" t="str">
         <v/>
@@ -5169,7 +5169,7 @@
         <v/>
       </c>
       <c r="H102">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I102" t="str">
         <v/>
@@ -5216,7 +5216,7 @@
         <v/>
       </c>
       <c r="H103">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I103" t="str">
         <v/>
@@ -5263,7 +5263,7 @@
         <v/>
       </c>
       <c r="H104">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="I104" t="str">
         <v/>
@@ -5310,7 +5310,7 @@
         <v/>
       </c>
       <c r="H105">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="I105" t="str">
         <v/>
@@ -5357,7 +5357,7 @@
         <v/>
       </c>
       <c r="H106">
-        <v>0</v>
+        <v>43</v>
       </c>
       <c r="I106" t="str">
         <v/>
@@ -5404,7 +5404,7 @@
         <v/>
       </c>
       <c r="H107">
-        <v>0</v>
+        <v>58</v>
       </c>
       <c r="I107" t="str">
         <v/>
@@ -5451,7 +5451,7 @@
         <v/>
       </c>
       <c r="H108">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I108" t="str">
         <v/>
@@ -5498,7 +5498,7 @@
         <v/>
       </c>
       <c r="H109">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="I109" t="str">
         <v/>
@@ -5545,7 +5545,7 @@
         <v/>
       </c>
       <c r="H110">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I110" t="str">
         <v/>
@@ -5592,7 +5592,7 @@
         <v/>
       </c>
       <c r="H111">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I111" t="str">
         <v/>
@@ -5639,7 +5639,7 @@
         <v/>
       </c>
       <c r="H112">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="I112" t="str">
         <v/>
@@ -5686,7 +5686,7 @@
         <v/>
       </c>
       <c r="H113">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="I113" t="str">
         <v/>
@@ -5733,7 +5733,7 @@
         <v/>
       </c>
       <c r="H114">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I114" t="str">
         <v/>
@@ -5780,7 +5780,7 @@
         <v/>
       </c>
       <c r="H115">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="I115" t="str">
         <v/>
@@ -5827,7 +5827,7 @@
         <v/>
       </c>
       <c r="H116">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="I116" t="str">
         <v/>
@@ -5874,7 +5874,7 @@
         <v/>
       </c>
       <c r="H117">
-        <v>0</v>
+        <v>157</v>
       </c>
       <c r="I117" t="str">
         <v/>
@@ -5921,7 +5921,7 @@
         <v/>
       </c>
       <c r="H118">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I118" t="str">
         <v/>
@@ -5968,7 +5968,7 @@
         <v/>
       </c>
       <c r="H119">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="I119" t="str">
         <v/>
@@ -6015,7 +6015,7 @@
         <v/>
       </c>
       <c r="H120">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I120" t="str">
         <v/>
@@ -6062,7 +6062,7 @@
         <v/>
       </c>
       <c r="H121">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I121" t="str">
         <v/>
@@ -6109,7 +6109,7 @@
         <v/>
       </c>
       <c r="H122">
-        <v>0</v>
+        <v>208</v>
       </c>
       <c r="I122" t="str">
         <v/>
@@ -6156,7 +6156,7 @@
         <v/>
       </c>
       <c r="H123">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I123" t="str">
         <v/>
@@ -6203,7 +6203,7 @@
         <v/>
       </c>
       <c r="H124">
-        <v>0</v>
+        <v>147</v>
       </c>
       <c r="I124" t="str">
         <v/>
@@ -6250,7 +6250,7 @@
         <v/>
       </c>
       <c r="H125">
-        <v>0</v>
+        <v>20.5</v>
       </c>
       <c r="I125" t="str">
         <v/>
@@ -6297,7 +6297,7 @@
         <v/>
       </c>
       <c r="H126">
-        <v>0</v>
+        <v>19.5</v>
       </c>
       <c r="I126" t="str">
         <v/>
@@ -6344,7 +6344,7 @@
         <v/>
       </c>
       <c r="H127">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="I127" t="str">
         <v/>
@@ -6391,7 +6391,7 @@
         <v/>
       </c>
       <c r="H128">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I128" t="str">
         <v/>
@@ -6438,7 +6438,7 @@
         <v/>
       </c>
       <c r="H129">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I129" t="str">
         <v/>
@@ -6485,7 +6485,7 @@
         <v/>
       </c>
       <c r="H130">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I130" t="str">
         <v/>
@@ -6532,7 +6532,7 @@
         <v/>
       </c>
       <c r="H131">
-        <v>0</v>
+        <v>285</v>
       </c>
       <c r="I131" t="str">
         <v/>
@@ -6579,7 +6579,7 @@
         <v/>
       </c>
       <c r="H132">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="I132" t="str">
         <v/>
@@ -6626,7 +6626,7 @@
         <v/>
       </c>
       <c r="H133">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="I133" t="str">
         <v/>
@@ -6673,7 +6673,7 @@
         <v/>
       </c>
       <c r="H134">
-        <v>0</v>
+        <v>131</v>
       </c>
       <c r="I134" t="str">
         <v/>
@@ -6720,7 +6720,7 @@
         <v/>
       </c>
       <c r="H135">
-        <v>0</v>
+        <v>94</v>
       </c>
       <c r="I135" t="str">
         <v/>
@@ -6767,7 +6767,7 @@
         <v/>
       </c>
       <c r="H136">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="I136" t="str">
         <v/>
@@ -6814,7 +6814,7 @@
         <v/>
       </c>
       <c r="H137">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="I137" t="str">
         <v/>
@@ -6861,7 +6861,7 @@
         <v/>
       </c>
       <c r="H138">
-        <v>0</v>
+        <v>124</v>
       </c>
       <c r="I138" t="str">
         <v/>
@@ -6908,7 +6908,7 @@
         <v/>
       </c>
       <c r="H139">
-        <v>0</v>
+        <v>143</v>
       </c>
       <c r="I139" t="str">
         <v/>
@@ -6955,7 +6955,7 @@
         <v/>
       </c>
       <c r="H140">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I140" t="str">
         <v/>
@@ -7002,7 +7002,7 @@
         <v/>
       </c>
       <c r="H141">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I141" t="str">
         <v/>
@@ -7049,7 +7049,7 @@
         <v/>
       </c>
       <c r="H142">
-        <v>0</v>
+        <v>490</v>
       </c>
       <c r="I142" t="str">
         <v/>
@@ -7096,7 +7096,7 @@
         <v/>
       </c>
       <c r="H143">
-        <v>0</v>
+        <v>143</v>
       </c>
       <c r="I143" t="str">
         <v/>
@@ -7143,7 +7143,7 @@
         <v/>
       </c>
       <c r="H144">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I144" t="str">
         <v/>
@@ -7190,7 +7190,7 @@
         <v/>
       </c>
       <c r="H145">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I145" t="str">
         <v/>
@@ -7237,7 +7237,7 @@
         <v/>
       </c>
       <c r="H146">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I146" t="str">
         <v/>
@@ -7284,7 +7284,7 @@
         <v/>
       </c>
       <c r="H147">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="I147" t="str">
         <v/>
@@ -7331,7 +7331,7 @@
         <v/>
       </c>
       <c r="H148">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I148" t="str">
         <v/>
@@ -7378,7 +7378,7 @@
         <v/>
       </c>
       <c r="H149">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I149" t="str">
         <v/>
@@ -7425,7 +7425,7 @@
         <v/>
       </c>
       <c r="H150">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I150" t="str">
         <v/>
@@ -7472,7 +7472,7 @@
         <v/>
       </c>
       <c r="H151">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I151" t="str">
         <v/>
@@ -7519,7 +7519,7 @@
         <v/>
       </c>
       <c r="H152">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I152" t="str">
         <v/>
@@ -7566,7 +7566,7 @@
         <v/>
       </c>
       <c r="H153">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I153" t="str">
         <v/>
@@ -7613,7 +7613,7 @@
         <v/>
       </c>
       <c r="H154">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I154" t="str">
         <v/>
@@ -7660,7 +7660,7 @@
         <v/>
       </c>
       <c r="H155">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I155" t="str">
         <v/>
@@ -7707,7 +7707,7 @@
         <v/>
       </c>
       <c r="H156">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I156" t="str">
         <v/>
@@ -7754,7 +7754,7 @@
         <v/>
       </c>
       <c r="H157">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I157" t="str">
         <v/>
@@ -7801,7 +7801,7 @@
         <v/>
       </c>
       <c r="H158">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I158" t="str">
         <v/>
@@ -7848,7 +7848,7 @@
         <v/>
       </c>
       <c r="H159">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I159" t="str">
         <v/>
@@ -7895,7 +7895,7 @@
         <v/>
       </c>
       <c r="H160">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I160" t="str">
         <v/>
@@ -8694,7 +8694,7 @@
         <v/>
       </c>
       <c r="H177">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I177" t="str">
         <v/>
@@ -8741,7 +8741,7 @@
         <v/>
       </c>
       <c r="H178">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I178" t="str">
         <v/>
@@ -8788,7 +8788,7 @@
         <v/>
       </c>
       <c r="H179">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I179" t="str">
         <v/>
@@ -8835,7 +8835,7 @@
         <v/>
       </c>
       <c r="H180">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I180" t="str">
         <v/>
@@ -8882,7 +8882,7 @@
         <v/>
       </c>
       <c r="H181">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I181" t="str">
         <v/>
@@ -8929,7 +8929,7 @@
         <v/>
       </c>
       <c r="H182">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I182" t="str">
         <v/>
@@ -8976,7 +8976,7 @@
         <v/>
       </c>
       <c r="H183">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I183" t="str">
         <v/>
@@ -9023,7 +9023,7 @@
         <v/>
       </c>
       <c r="H184">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I184" t="str">
         <v/>
@@ -9070,7 +9070,7 @@
         <v/>
       </c>
       <c r="H185">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I185" t="str">
         <v/>
@@ -9117,7 +9117,7 @@
         <v/>
       </c>
       <c r="H186">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I186" t="str">
         <v/>
@@ -9164,7 +9164,7 @@
         <v/>
       </c>
       <c r="H187">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I187" t="str">
         <v/>
@@ -9211,7 +9211,7 @@
         <v/>
       </c>
       <c r="H188">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I188" t="str">
         <v/>
@@ -9258,7 +9258,7 @@
         <v/>
       </c>
       <c r="H189">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I189" t="str">
         <v/>
@@ -9305,7 +9305,7 @@
         <v/>
       </c>
       <c r="H190">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="I190" t="str">
         <v/>
@@ -9352,7 +9352,7 @@
         <v/>
       </c>
       <c r="H191">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I191" t="str">
         <v/>
@@ -9399,7 +9399,7 @@
         <v/>
       </c>
       <c r="H192">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I192" t="str">
         <v/>
@@ -9446,7 +9446,7 @@
         <v/>
       </c>
       <c r="H193">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I193" t="str">
         <v/>
@@ -9493,7 +9493,7 @@
         <v/>
       </c>
       <c r="H194">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I194" t="str">
         <v/>
@@ -9540,7 +9540,7 @@
         <v/>
       </c>
       <c r="H195">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="I195" t="str">
         <v/>
@@ -10386,7 +10386,7 @@
         <v/>
       </c>
       <c r="H213">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I213" t="str">
         <v/>
@@ -10433,7 +10433,7 @@
         <v/>
       </c>
       <c r="H214">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I214" t="str">
         <v/>
@@ -10480,7 +10480,7 @@
         <v/>
       </c>
       <c r="H215">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I215" t="str">
         <v/>
@@ -10527,7 +10527,7 @@
         <v/>
       </c>
       <c r="H216">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I216" t="str">
         <v/>
@@ -10574,7 +10574,7 @@
         <v/>
       </c>
       <c r="H217">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="I217" t="str">
         <v/>
@@ -10621,7 +10621,7 @@
         <v/>
       </c>
       <c r="H218">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I218" t="str">
         <v/>
@@ -10668,7 +10668,7 @@
         <v/>
       </c>
       <c r="H219">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I219" t="str">
         <v/>
@@ -10715,7 +10715,7 @@
         <v/>
       </c>
       <c r="H220">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I220" t="str">
         <v/>
@@ -10762,7 +10762,7 @@
         <v/>
       </c>
       <c r="H221">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I221" t="str">
         <v/>
@@ -10809,7 +10809,7 @@
         <v/>
       </c>
       <c r="H222">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I222" t="str">
         <v/>
@@ -10856,7 +10856,7 @@
         <v/>
       </c>
       <c r="H223">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I223" t="str">
         <v/>
@@ -10903,7 +10903,7 @@
         <v/>
       </c>
       <c r="H224">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I224" t="str">
         <v/>
@@ -10950,7 +10950,7 @@
         <v/>
       </c>
       <c r="H225">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I225" t="str">
         <v/>
@@ -10997,7 +10997,7 @@
         <v/>
       </c>
       <c r="H226">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I226" t="str">
         <v/>
@@ -11044,7 +11044,7 @@
         <v/>
       </c>
       <c r="H227">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I227" t="str">
         <v/>
@@ -11091,7 +11091,7 @@
         <v/>
       </c>
       <c r="H228">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="I228" t="str">
         <v/>
@@ -11138,7 +11138,7 @@
         <v/>
       </c>
       <c r="H229">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I229" t="str">
         <v/>
@@ -11185,7 +11185,7 @@
         <v/>
       </c>
       <c r="H230">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="I230" t="str">
         <v/>
@@ -11232,7 +11232,7 @@
         <v/>
       </c>
       <c r="H231">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I231" t="str">
         <v/>
@@ -11279,7 +11279,7 @@
         <v/>
       </c>
       <c r="H232">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I232" t="str">
         <v/>
@@ -11326,7 +11326,7 @@
         <v/>
       </c>
       <c r="H233">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I233" t="str">
         <v/>
@@ -13018,7 +13018,7 @@
         <v/>
       </c>
       <c r="H269">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="I269" t="str">
         <v/>
@@ -13065,7 +13065,7 @@
         <v/>
       </c>
       <c r="H270">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I270" t="str">
         <v/>
@@ -13112,7 +13112,7 @@
         <v/>
       </c>
       <c r="H271">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I271" t="str">
         <v/>
@@ -13159,7 +13159,7 @@
         <v/>
       </c>
       <c r="H272">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="I272" t="str">
         <v/>
@@ -13206,7 +13206,7 @@
         <v/>
       </c>
       <c r="H273">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I273" t="str">
         <v/>
@@ -13253,7 +13253,7 @@
         <v/>
       </c>
       <c r="H274">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I274" t="str">
         <v/>
@@ -13300,7 +13300,7 @@
         <v/>
       </c>
       <c r="H275">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I275" t="str">
         <v/>
@@ -13347,7 +13347,7 @@
         <v/>
       </c>
       <c r="H276">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="I276" t="str">
         <v/>
@@ -13394,7 +13394,7 @@
         <v/>
       </c>
       <c r="H277">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I277" t="str">
         <v/>
@@ -13441,7 +13441,7 @@
         <v/>
       </c>
       <c r="H278">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="I278" t="str">
         <v/>
@@ -13488,7 +13488,7 @@
         <v/>
       </c>
       <c r="H279">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I279" t="str">
         <v/>
@@ -13535,7 +13535,7 @@
         <v/>
       </c>
       <c r="H280">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I280" t="str">
         <v/>
@@ -13582,7 +13582,7 @@
         <v/>
       </c>
       <c r="H281">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="I281" t="str">
         <v/>
@@ -15086,7 +15086,7 @@
         <v/>
       </c>
       <c r="H313">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I313" t="str">
         <v/>
@@ -15133,7 +15133,7 @@
         <v/>
       </c>
       <c r="H314">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I314" t="str">
         <v/>
@@ -15180,7 +15180,7 @@
         <v/>
       </c>
       <c r="H315">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I315" t="str">
         <v/>
@@ -15227,7 +15227,7 @@
         <v/>
       </c>
       <c r="H316">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I316" t="str">
         <v/>
@@ -15274,7 +15274,7 @@
         <v/>
       </c>
       <c r="H317">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I317" t="str">
         <v/>
@@ -15321,7 +15321,7 @@
         <v/>
       </c>
       <c r="H318">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I318" t="str">
         <v/>
@@ -15368,7 +15368,7 @@
         <v/>
       </c>
       <c r="H319">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="I319" t="str">
         <v/>
@@ -15415,7 +15415,7 @@
         <v/>
       </c>
       <c r="H320">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I320" t="str">
         <v/>
@@ -15462,7 +15462,7 @@
         <v/>
       </c>
       <c r="H321">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I321" t="str">
         <v/>
@@ -15509,7 +15509,7 @@
         <v/>
       </c>
       <c r="H322">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I322" t="str">
         <v/>
@@ -15556,7 +15556,7 @@
         <v/>
       </c>
       <c r="H323">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I323" t="str">
         <v/>
@@ -15603,7 +15603,7 @@
         <v/>
       </c>
       <c r="H324">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I324" t="str">
         <v/>
@@ -15650,7 +15650,7 @@
         <v/>
       </c>
       <c r="H325">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I325" t="str">
         <v/>
@@ -15697,7 +15697,7 @@
         <v/>
       </c>
       <c r="H326">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I326" t="str">
         <v/>
@@ -15744,7 +15744,7 @@
         <v/>
       </c>
       <c r="H327">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I327" t="str">
         <v/>
@@ -15791,7 +15791,7 @@
         <v/>
       </c>
       <c r="H328">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I328" t="str">
         <v/>
@@ -15838,7 +15838,7 @@
         <v/>
       </c>
       <c r="H329">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="I329" t="str">
         <v/>
@@ -15885,7 +15885,7 @@
         <v/>
       </c>
       <c r="H330">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I330" t="str">
         <v/>
@@ -16590,7 +16590,7 @@
         <v/>
       </c>
       <c r="H345">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I345" t="str">
         <v/>
@@ -18047,7 +18047,7 @@
         <v/>
       </c>
       <c r="H376">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="I376" t="str">
         <v/>
@@ -18470,7 +18470,7 @@
         <v/>
       </c>
       <c r="H385">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="I385" t="str">
         <v/>

</xml_diff>